<commit_message>
commit de chuyen nhanh
</commit_message>
<xml_diff>
--- a/backend/unit_test/quanlytaikhoan/fileTest/ds-test-sai-dinh-dang.xlsx
+++ b/backend/unit_test/quanlytaikhoan/fileTest/ds-test-sai-dinh-dang.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ThucTapTotNghiep\QuanLyLopHoc\backend\unit_test\quanlytaikhoan\fileTest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A22DC41-37EB-4378-9CFD-425B9F10B41D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{740BC4FC-D006-4FFD-B9EB-E9B2D94D85DE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8988" xr2:uid="{313CC9A6-8821-4C61-BBE4-183FB7BFBE31}"/>
   </bookViews>
@@ -78,13 +78,13 @@
     <t>D22_TH10</t>
   </si>
   <si>
-    <t>DH52200320@student.stu.edu.vn</t>
-  </si>
-  <si>
     <t>Trần Quốc</t>
   </si>
   <si>
     <t>DH5220032021</t>
+  </si>
+  <si>
+    <t>DH52200320student.stu.edu.vn</t>
   </si>
 </sst>
 </file>
@@ -2040,12 +2040,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>15</v>
@@ -2059,7 +2059,7 @@
       <c r="F2" s="6"/>
       <c r="G2" s="4"/>
       <c r="H2" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I2" s="6"/>
     </row>
@@ -2071,7 +2071,7 @@
         <v>13</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>9</v>

</xml_diff>